<commit_message>
fix: realistic test data — bank stmt has old+new+debits mixed
Bank statement now contains 28 transactions:
- 10 OLD transactions matching master sheet refs (agent should SKIP)
- 3 bank charge debits (agent should SKIP)
- 15 NEW Q1/Q2 installments (agent must detect, match, ADD to master)

This tests the full workflow: identify missing → match → update master

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/test_data/CBC_Escrow_Statement_Mar2026.xlsx
+++ b/test_data/CBC_Escrow_Statement_Mar2026.xlsx
@@ -443,12 +443,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G16"/>
+  <dimension ref="A1:G29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="70" customWidth="1" min="3" max="3"/>
+    <col width="75" customWidth="1" min="3" max="3"/>
     <col width="25" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
@@ -494,407 +494,758 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46095</v>
+        <v>46027</v>
       </c>
       <c r="B2" s="2" t="n">
-        <v>46095</v>
+        <v>46027</v>
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>INWARD REMITTANCETT REF: 530P4F86D98E301 AED 56250 AHMED HASSAN AL MAKTOUM PO BOX 12345 DUBAI UAE</t>
+          <t>OUTWARD CLEARINGUNIT 101 DEFAULT - ~026ABC001</t>
         </is>
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
-          <t>STMT-301</t>
+          <t>REF-H001</t>
         </is>
       </c>
       <c r="E2" s="4" t="n">
         <v>0</v>
       </c>
       <c r="F2" s="4" t="n">
-        <v>56250</v>
+        <v>450000</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>8556250</v>
+        <v>5450000</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>46096</v>
+        <v>46030</v>
       </c>
       <c r="B3" s="2" t="n">
-        <v>46096</v>
+        <v>46030</v>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>OUTWARD CLEARINGUNIT 102 DEFAULT - ~026STU901</t>
+          <t>INWARD REMITTANCETT REF: 530P4F86D98E100 AED 380000 FATIMA ABDULRAHMAN SAEED PO BOX 5432 DUBAI</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>STMT-302</t>
+          <t>REF-H002</t>
         </is>
       </c>
       <c r="E3" s="4" t="n">
         <v>0</v>
       </c>
       <c r="F3" s="4" t="n">
-        <v>47500</v>
+        <v>380000</v>
       </c>
       <c r="G3" s="4" t="n">
-        <v>8603750</v>
+        <v>5830000</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>46097</v>
+        <v>46034</v>
       </c>
       <c r="B4" s="2" t="n">
-        <v>46097</v>
+        <v>46034</v>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>INWARD REMITTANCETT REF: 033DBLC2608235 AED 65000 MOHAMED KHALID RASHIDI CIT YWALK BUILDING DUBAI</t>
+          <t>OUTWARD CLEARINGUNIT 203 DEFAULT - ~026ABC003</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>STMT-303</t>
+          <t>REF-H003</t>
         </is>
       </c>
       <c r="E4" s="4" t="n">
         <v>0</v>
       </c>
       <c r="F4" s="4" t="n">
-        <v>65000</v>
+        <v>520000</v>
       </c>
       <c r="G4" s="4" t="n">
-        <v>8668750</v>
+        <v>6350000</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>46098</v>
+        <v>46037</v>
       </c>
       <c r="B5" s="2" t="n">
-        <v>46098</v>
+        <v>46037</v>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>IPP Customer CreditIPP 20260317ADC6B981204</t>
+          <t>INWARD REMITTANCETT REF: 044ABLC7890100 AED 490000 SARAH JOHNSON 45 PARK LANE LONDON</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>STMT-304</t>
+          <t>REF-H004</t>
         </is>
       </c>
       <c r="E5" s="4" t="n">
         <v>0</v>
       </c>
       <c r="F5" s="4" t="n">
-        <v>61250</v>
+        <v>490000</v>
       </c>
       <c r="G5" s="4" t="n">
-        <v>8730000</v>
+        <v>6840000</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>46099</v>
+        <v>46042</v>
       </c>
       <c r="B6" s="2" t="n">
-        <v>46099</v>
+        <v>46042</v>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>INWARD REMITTANCETT REF: 20260318004944 AED 51250 KH OMAR AL MANSOURI</t>
+          <t>OUTWARD CLEARINGUNIT 305 DEFAULT - ~026ABC005</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>STMT-305</t>
+          <t>REF-H005</t>
         </is>
       </c>
       <c r="E6" s="4" t="n">
         <v>0</v>
       </c>
       <c r="F6" s="4" t="n">
-        <v>51250</v>
+        <v>410000</v>
       </c>
       <c r="G6" s="4" t="n">
-        <v>8781250</v>
+        <v>7250000</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
-        <v>46100</v>
+        <v>46047</v>
       </c>
       <c r="B7" s="2" t="n">
-        <v>46100</v>
+        <v>46047</v>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>OUTWARD CLEARINGUNIT 306 DEFAULT - ~026VWX234</t>
+          <t>INWARD REMITTANCETT REF: 20260125001000 AED 375000 NADIA HASSAN IBRAHIM</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>STMT-306</t>
+          <t>REF-H006</t>
         </is>
       </c>
       <c r="E7" s="4" t="n">
         <v>0</v>
       </c>
       <c r="F7" s="4" t="n">
-        <v>46875</v>
+        <v>375000</v>
       </c>
       <c r="G7" s="4" t="n">
-        <v>8828125</v>
+        <v>7625000</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
-        <v>46101</v>
+        <v>46054</v>
       </c>
       <c r="B8" s="2" t="n">
-        <v>46101</v>
+        <v>46054</v>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>INWARD REMITTANCETT REF: 530P5EB4FCD5BB AED 70000 RASHID SAEED ALKETBI</t>
+          <t>OUTWARD CLEARINGUNIT 407 DEFAULT - ~026ABC007</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>STMT-307</t>
+          <t>REF-H007</t>
         </is>
       </c>
       <c r="E8" s="4" t="n">
         <v>0</v>
       </c>
       <c r="F8" s="4" t="n">
-        <v>70000</v>
+        <v>560000</v>
       </c>
       <c r="G8" s="4" t="n">
-        <v>8898125</v>
+        <v>8185000</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
-        <v>46102</v>
+        <v>46058</v>
       </c>
       <c r="B9" s="2" t="n">
-        <v>46102</v>
+        <v>46058</v>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>INWARD REMITTANCETT REF: 044ABLC1234567 AED 53750 ELENA PETROVNA MOSCOW RUSSIA</t>
+          <t>INWARD REMITTANCETT REF: 530P5EB4FCD500 AED 430000 ELENA PETROVA MOSCOW RUSSIA</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>STMT-308</t>
+          <t>REF-H008</t>
         </is>
       </c>
       <c r="E9" s="4" t="n">
         <v>0</v>
       </c>
       <c r="F9" s="4" t="n">
-        <v>53750</v>
+        <v>430000</v>
       </c>
       <c r="G9" s="4" t="n">
-        <v>8951875</v>
+        <v>8615000</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
-        <v>46103</v>
+        <v>46063</v>
       </c>
       <c r="B10" s="2" t="n">
-        <v>46103</v>
+        <v>46063</v>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>INWARD REMITTANCETT REF: 20260322123456 AED 63750 A M AL SUWAIDI</t>
+          <t>OUTWARD CLEARINGUNIT 509 DEFAULT - ~026ABC009</t>
         </is>
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>STMT-309</t>
+          <t>REF-H009</t>
         </is>
       </c>
       <c r="E10" s="4" t="n">
         <v>0</v>
       </c>
       <c r="F10" s="4" t="n">
-        <v>63750</v>
+        <v>510000</v>
       </c>
       <c r="G10" s="4" t="n">
-        <v>9015625</v>
+        <v>9125000</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
-        <v>46103</v>
+        <v>46068</v>
       </c>
       <c r="B11" s="2" t="n">
-        <v>46103</v>
+        <v>46068</v>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>OUTWARD CLEARINGUNIT 510 DEFAULT - ~026YZA567</t>
+          <t>INWARD REMITTANCETT REF: 20260215005000 AED 395000 JAMES ROBERT WILSON FLAT 12 CHICAGO</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>STMT-310</t>
+          <t>REF-H010</t>
         </is>
       </c>
       <c r="E11" s="4" t="n">
         <v>0</v>
       </c>
       <c r="F11" s="4" t="n">
-        <v>49375</v>
+        <v>395000</v>
       </c>
       <c r="G11" s="4" t="n">
-        <v>9065000</v>
+        <v>9520000</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
-        <v>46104</v>
+        <v>46073</v>
       </c>
       <c r="B12" s="2" t="n">
-        <v>46104</v>
+        <v>46073</v>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>INWARD REMITTANCETT REF: 789ABC123DEF AED 56250 AHMED H MAKTOUM</t>
+          <t>BANK CHARGES - MONTHLY FEE</t>
         </is>
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>STMT-311</t>
+          <t>REF-BANK01</t>
         </is>
       </c>
       <c r="E12" s="4" t="n">
-        <v>0</v>
+        <v>1500</v>
       </c>
       <c r="F12" s="4" t="n">
-        <v>56250</v>
+        <v>0</v>
       </c>
       <c r="G12" s="4" t="n">
-        <v>9121250</v>
+        <v>9518500</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
-        <v>46105</v>
+        <v>46082</v>
       </c>
       <c r="B13" s="2" t="n">
-        <v>46105</v>
+        <v>46082</v>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>INWARD REMITTANCETT REF: 456DEF789GHI AED 47500 FATIMA SAEED</t>
+          <t>SWIFT CHARGES - INWARD REMITTANCE</t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>STMT-312</t>
+          <t>REF-BANK02</t>
         </is>
       </c>
       <c r="E13" s="4" t="n">
-        <v>0</v>
+        <v>250</v>
       </c>
       <c r="F13" s="4" t="n">
-        <v>47500</v>
+        <v>0</v>
       </c>
       <c r="G13" s="4" t="n">
-        <v>9168750</v>
+        <v>9518250</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
-        <v>46105</v>
+        <v>46091</v>
       </c>
       <c r="B14" s="2" t="n">
-        <v>46105</v>
+        <v>46091</v>
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>BANKNET AE420350000000123456789 12345678 MOHAMMED K AL RASHIDI</t>
+          <t>BANK CHARGES - STATEMENT FEE</t>
         </is>
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>STMT-313</t>
+          <t>REF-BANK03</t>
         </is>
       </c>
       <c r="E14" s="4" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="F14" s="4" t="n">
-        <v>65000</v>
+        <v>0</v>
       </c>
       <c r="G14" s="4" t="n">
-        <v>9233750</v>
+        <v>9518150</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
-        <v>46106</v>
+        <v>46095</v>
       </c>
       <c r="B15" s="2" t="n">
-        <v>46106</v>
+        <v>46095</v>
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>INWARD REMITTANCETT REF: 111222333444 AED 46875 NADIA IBRAHIM</t>
+          <t>INWARD REMITTANCETT REF: 530P4F86D98E301 AED 56250 AHMED HASSAN AL MAKTOUM PO BOX 12345 DUBAI UAE</t>
         </is>
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>STMT-314</t>
+          <t>STMT-301</t>
         </is>
       </c>
       <c r="E15" s="4" t="n">
         <v>0</v>
       </c>
       <c r="F15" s="4" t="n">
-        <v>46875</v>
+        <v>56250</v>
       </c>
       <c r="G15" s="4" t="n">
-        <v>9280625</v>
+        <v>9574400</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
+        <v>46096</v>
+      </c>
+      <c r="B16" s="2" t="n">
+        <v>46096</v>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>OUTWARD CLEARINGUNIT 102 DEFAULT - ~026STU901</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>STMT-302</t>
+        </is>
+      </c>
+      <c r="E16" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F16" s="4" t="n">
+        <v>47500</v>
+      </c>
+      <c r="G16" s="4" t="n">
+        <v>9621900</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="n">
+        <v>46097</v>
+      </c>
+      <c r="B17" s="2" t="n">
+        <v>46097</v>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>INWARD REMITTANCETT REF: 033DBLC2608235 AED 65000 MOHAMED KHALID RASHIDI CIT YWALK BUILDING DUBAI</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>STMT-303</t>
+        </is>
+      </c>
+      <c r="E17" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F17" s="4" t="n">
+        <v>65000</v>
+      </c>
+      <c r="G17" s="4" t="n">
+        <v>9686900</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="n">
+        <v>46098</v>
+      </c>
+      <c r="B18" s="2" t="n">
+        <v>46098</v>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>IPP Customer CreditIPP 20260317ADC6B981204</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>STMT-304</t>
+        </is>
+      </c>
+      <c r="E18" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F18" s="4" t="n">
+        <v>61250</v>
+      </c>
+      <c r="G18" s="4" t="n">
+        <v>9748150</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="n">
+        <v>46099</v>
+      </c>
+      <c r="B19" s="2" t="n">
+        <v>46099</v>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>INWARD REMITTANCETT REF: 20260318004944 AED 51250 KH OMAR AL MANSOURI</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>STMT-305</t>
+        </is>
+      </c>
+      <c r="E19" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F19" s="4" t="n">
+        <v>51250</v>
+      </c>
+      <c r="G19" s="4" t="n">
+        <v>9799400</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="n">
+        <v>46100</v>
+      </c>
+      <c r="B20" s="2" t="n">
+        <v>46100</v>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>OUTWARD CLEARINGUNIT 306 DEFAULT - ~026VWX234</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>STMT-306</t>
+        </is>
+      </c>
+      <c r="E20" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F20" s="4" t="n">
+        <v>46875</v>
+      </c>
+      <c r="G20" s="4" t="n">
+        <v>9846275</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="n">
+        <v>46101</v>
+      </c>
+      <c r="B21" s="2" t="n">
+        <v>46101</v>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>INWARD REMITTANCETT REF: 530P5EB4FCD5BB AED 70000 RASHID SAEED ALKETBI</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>STMT-307</t>
+        </is>
+      </c>
+      <c r="E21" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F21" s="4" t="n">
+        <v>70000</v>
+      </c>
+      <c r="G21" s="4" t="n">
+        <v>9916275</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="n">
+        <v>46102</v>
+      </c>
+      <c r="B22" s="2" t="n">
+        <v>46102</v>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>INWARD REMITTANCETT REF: 044ABLC1234567 AED 53750 ELENA PETROVNA MOSCOW RUSSIA</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>STMT-308</t>
+        </is>
+      </c>
+      <c r="E22" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F22" s="4" t="n">
+        <v>53750</v>
+      </c>
+      <c r="G22" s="4" t="n">
+        <v>9970025</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="n">
+        <v>46103</v>
+      </c>
+      <c r="B23" s="2" t="n">
+        <v>46103</v>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>INWARD REMITTANCETT REF: 20260322123456 AED 63750 A M AL SUWAIDI</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>STMT-309</t>
+        </is>
+      </c>
+      <c r="E23" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F23" s="4" t="n">
+        <v>63750</v>
+      </c>
+      <c r="G23" s="4" t="n">
+        <v>10033775</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="n">
+        <v>46103</v>
+      </c>
+      <c r="B24" s="2" t="n">
+        <v>46103</v>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>OUTWARD CLEARINGUNIT 510 DEFAULT - ~026YZA567</t>
+        </is>
+      </c>
+      <c r="D24" s="3" t="inlineStr">
+        <is>
+          <t>STMT-310</t>
+        </is>
+      </c>
+      <c r="E24" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F24" s="4" t="n">
+        <v>49375</v>
+      </c>
+      <c r="G24" s="4" t="n">
+        <v>10083150</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="n">
+        <v>46104</v>
+      </c>
+      <c r="B25" s="2" t="n">
+        <v>46104</v>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>INWARD REMITTANCETT REF: 789ABC123DEF01 AED 56250 AHMED H MAKTOUM</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="inlineStr">
+        <is>
+          <t>STMT-311</t>
+        </is>
+      </c>
+      <c r="E25" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F25" s="4" t="n">
+        <v>56250</v>
+      </c>
+      <c r="G25" s="4" t="n">
+        <v>10139400</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="n">
+        <v>46105</v>
+      </c>
+      <c r="B26" s="2" t="n">
+        <v>46105</v>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>INWARD REMITTANCETT REF: 456DEF789GHI02 AED 47500 FATIMA SAEED</t>
+        </is>
+      </c>
+      <c r="D26" s="3" t="inlineStr">
+        <is>
+          <t>STMT-312</t>
+        </is>
+      </c>
+      <c r="E26" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F26" s="4" t="n">
+        <v>47500</v>
+      </c>
+      <c r="G26" s="4" t="n">
+        <v>10186900</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="n">
+        <v>46105</v>
+      </c>
+      <c r="B27" s="2" t="n">
+        <v>46105</v>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>BANKNET AE420350000000123456789 12345678 MOHAMMED K AL RASHIDI</t>
+        </is>
+      </c>
+      <c r="D27" s="3" t="inlineStr">
+        <is>
+          <t>STMT-313</t>
+        </is>
+      </c>
+      <c r="E27" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F27" s="4" t="n">
+        <v>65000</v>
+      </c>
+      <c r="G27" s="4" t="n">
+        <v>10251900</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="n">
+        <v>46106</v>
+      </c>
+      <c r="B28" s="2" t="n">
+        <v>46106</v>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>INWARD REMITTANCETT REF: 111222333444 AED 46875 NADIA IBRAHIM</t>
+        </is>
+      </c>
+      <c r="D28" s="3" t="inlineStr">
+        <is>
+          <t>STMT-314</t>
+        </is>
+      </c>
+      <c r="E28" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F28" s="4" t="n">
+        <v>46875</v>
+      </c>
+      <c r="G28" s="4" t="n">
+        <v>10298775</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="n">
         <v>46107</v>
       </c>
-      <c r="B16" s="2" t="n">
+      <c r="B29" s="2" t="n">
         <v>46107</v>
       </c>
-      <c r="C16" s="3" t="inlineStr">
+      <c r="C29" s="3" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="D16" s="3" t="inlineStr">
+      <c r="D29" s="3" t="inlineStr">
         <is>
           <t>STMT-315</t>
         </is>
       </c>
-      <c r="E16" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="F16" s="4" t="n">
+      <c r="E29" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F29" s="4" t="n">
         <v>51250</v>
       </c>
-      <c r="G16" s="4" t="n">
-        <v>9331875</v>
+      <c r="G29" s="4" t="n">
+        <v>10350025</v>
       </c>
     </row>
   </sheetData>

</xml_diff>